<commit_message>
Add doughnut alternative for channel composition
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0122Czh11joCd8pnuPmWyXv4
</commit_message>
<xml_diff>
--- a/lab02/APIO114_Lab02_2713963.xlsx
+++ b/lab02/APIO114_Lab02_2713963.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Dashboard" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">Dashboard!$A$1:$T$22</definedName>
+    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Area" vbProcedure="false">Dashboard!$A$1:$AC$22</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="78">
   <si>
     <t xml:space="preserve">Lab 2 Chart Choice and Visual Design</t>
   </si>
@@ -179,6 +179,9 @@
     <t xml:space="preserve">Orders: channels</t>
   </si>
   <si>
+    <t xml:space="preserve">Channel (largest first)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Design decision</t>
   </si>
   <si>
@@ -212,6 +215,12 @@
     <t xml:space="preserve">Chart 2 Revenue by channel</t>
   </si>
   <si>
+    <t xml:space="preserve">Chart 2 alternative – doughnut (backup)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part-to-whole confirmed (channels = 100% of revenue, 480 orders). The doughnut is kept for reference: all three channels, slices sorted largest first from 12 o'clock, % labels on the slices, one highlight color, no gradient, 3D or exploded slices. Because the slices are nearly equal, the sorted bar chart is the main Chart 2.</t>
+  </si>
+  <si>
     <t xml:space="preserve">The data is part-to-whole: the three channels add up to the same total as the categories (SAR 35,467) and every order belongs to one channel (3 × 160 = 480 orders). However, the shares are very close (35.4%, 33.4%, 31.2%), so doughnut slices would look almost equal and be hard to compare. Following the lab rule, a sorted bar chart of percentage share was used instead of a doughnut.</t>
   </si>
   <si>
@@ -251,7 +260,7 @@
     <t xml:space="preserve">APIO 114 – Lab 2 Chart Choice and Visual Design  |  Student ID 2713963</t>
   </si>
   <si>
-    <t xml:space="preserve">Final corrected charts: category comparison and channel composition</t>
+    <t xml:space="preserve">Final corrected charts: category comparison, channel composition (sorted bar) and doughnut alternative for reference</t>
   </si>
 </sst>
 </file>
@@ -391,7 +400,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDEBF7"/>
-        <bgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFD5DCE6"/>
       </patternFill>
     </fill>
   </fills>
@@ -527,12 +536,12 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
@@ -577,7 +586,7 @@
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF1F5C8B"/>
-      <rgbColor rgb="FFD0D0D0"/>
+      <rgbColor rgb="FFD5DCE6"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -593,14 +602,14 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFD0D0D0"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF4F81BD"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF1B365D"/>
       <rgbColor rgb="FF339966"/>
@@ -798,11 +807,11 @@
         </c:ser>
         <c:gapWidth val="55"/>
         <c:overlap val="0"/>
-        <c:axId val="9025491"/>
-        <c:axId val="11033005"/>
+        <c:axId val="32317593"/>
+        <c:axId val="23578775"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="9025491"/>
+        <c:axId val="32317593"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -834,7 +843,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11033005"/>
+        <c:crossAx val="23578775"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -842,7 +851,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11033005"/>
+        <c:axId val="23578775"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -909,7 +918,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9025491"/>
+        <c:crossAx val="32317593"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1114,11 +1123,11 @@
         </c:ser>
         <c:gapWidth val="55"/>
         <c:overlap val="0"/>
-        <c:axId val="6158267"/>
-        <c:axId val="23420973"/>
+        <c:axId val="30973237"/>
+        <c:axId val="717923"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="6158267"/>
+        <c:axId val="30973237"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1150,7 +1159,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23420973"/>
+        <c:crossAx val="717923"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1158,7 +1167,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="23420973"/>
+        <c:axId val="717923"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1225,7 +1234,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6158267"/>
+        <c:crossAx val="30973237"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1254,6 +1263,273 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Revenue share by channel</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Chart Workspace'!K19</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Revenue SAR</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4f81bd"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:explosion val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1f5c8b"/>
+              </a:solidFill>
+              <a:ln w="19080">
+                <a:solidFill>
+                  <a:srgbClr val="ffffff"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="a9b7c9"/>
+              </a:solidFill>
+              <a:ln w="19080">
+                <a:solidFill>
+                  <a:srgbClr val="ffffff"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="d5dce6"/>
+              </a:solidFill>
+              <a:ln w="19080">
+                <a:solidFill>
+                  <a:srgbClr val="ffffff"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:txPr>
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                      <a:latin typeface="Calibri"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="1"/>
+              <c:separator>
+</c:separator>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:txPr>
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                      <a:latin typeface="Calibri"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="1"/>
+              <c:separator>
+</c:separator>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:txPr>
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                      <a:latin typeface="Calibri"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="1"/>
+              <c:separator>
+</c:separator>
+            </c:dLbl>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:separator>
+</c:separator>
+            <c:showLeaderLines val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Chart Workspace'!$J$20:$J$22</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Click and Collect</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Delivery</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>In Store</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Chart Workspace'!$K$20:$K$22</c:f>
+              <c:numCache>
+                <c:formatCode>"SAR "#,##0</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>12557</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11838</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11072</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="50"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -1384,11 +1660,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="13383268"/>
-        <c:axId val="19956579"/>
+        <c:axId val="82262247"/>
+        <c:axId val="81605395"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="13383268"/>
+        <c:axId val="82262247"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1420,7 +1696,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19956579"/>
+        <c:crossAx val="81605395"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1428,7 +1704,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19956579"/>
+        <c:axId val="81605395"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13000"/>
@@ -1472,7 +1748,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13383268"/>
+        <c:crossAx val="82262247"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1500,7 +1776,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -1677,11 +1953,11 @@
         </c:ser>
         <c:gapWidth val="55"/>
         <c:overlap val="0"/>
-        <c:axId val="88628349"/>
-        <c:axId val="67840449"/>
+        <c:axId val="93270546"/>
+        <c:axId val="44166114"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="88628349"/>
+        <c:axId val="93270546"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1713,7 +1989,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="67840449"/>
+        <c:crossAx val="44166114"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1721,7 +1997,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="67840449"/>
+        <c:axId val="44166114"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1788,7 +2064,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88628349"/>
+        <c:crossAx val="93270546"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1816,7 +2092,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -1999,11 +2275,11 @@
         </c:ser>
         <c:gapWidth val="55"/>
         <c:overlap val="0"/>
-        <c:axId val="16235296"/>
-        <c:axId val="43559666"/>
+        <c:axId val="62049311"/>
+        <c:axId val="35964258"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="16235296"/>
+        <c:axId val="62049311"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2035,7 +2311,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43559666"/>
+        <c:crossAx val="35964258"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2043,7 +2319,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="43559666"/>
+        <c:axId val="35964258"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2110,7 +2386,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16235296"/>
+        <c:crossAx val="62049311"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2138,7 +2414,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -2315,11 +2591,11 @@
         </c:ser>
         <c:gapWidth val="55"/>
         <c:overlap val="0"/>
-        <c:axId val="26664629"/>
-        <c:axId val="7341642"/>
+        <c:axId val="98401865"/>
+        <c:axId val="59230428"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="26664629"/>
+        <c:axId val="98401865"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2351,7 +2627,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7341642"/>
+        <c:crossAx val="59230428"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2359,7 +2635,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="7341642"/>
+        <c:axId val="59230428"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2426,10 +2702,277 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26664629"/>
+        <c:crossAx val="98401865"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Doughnut alternative: shares are nearly equal</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Chart Workspace'!K19</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Revenue SAR</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4f81bd"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:explosion val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1f5c8b"/>
+              </a:solidFill>
+              <a:ln w="19080">
+                <a:solidFill>
+                  <a:srgbClr val="ffffff"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="a9b7c9"/>
+              </a:solidFill>
+              <a:ln w="19080">
+                <a:solidFill>
+                  <a:srgbClr val="ffffff"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="d5dce6"/>
+              </a:solidFill>
+              <a:ln w="19080">
+                <a:solidFill>
+                  <a:srgbClr val="ffffff"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:txPr>
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                      <a:latin typeface="Calibri"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="1"/>
+              <c:separator>
+</c:separator>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:txPr>
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                      <a:latin typeface="Calibri"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="1"/>
+              <c:separator>
+</c:separator>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:txPr>
+                <a:bodyPr wrap="square"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
+                      <a:latin typeface="Calibri"/>
+                    </a:defRPr>
+                  </a:pPr>
+                </a:p>
+              </c:txPr>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="1"/>
+              <c:separator>
+</c:separator>
+            </c:dLbl>
+            <c:txPr>
+              <a:bodyPr wrap="square"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="Calibri"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:separator>
+</c:separator>
+            <c:showLeaderLines val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Chart Workspace'!$J$20:$J$22</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Click and Collect</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Delivery</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>In Store</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Chart Workspace'!$K$20:$K$22</c:f>
+              <c:numCache>
+                <c:formatCode>"SAR "#,##0</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>12557</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11838</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11072</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="50"/>
+      </c:doughnutChart>
       <c:spPr>
         <a:noFill/>
         <a:ln w="0">
@@ -2490,14 +3033,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>78120</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>128520</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>32760</xdr:rowOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>110880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2518,16 +3061,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>78120</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>128520</xdr:colOff>
-      <xdr:row>65</xdr:row>
-      <xdr:rowOff>32760</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>231840</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>110880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2535,8 +3078,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="0" y="14725800"/>
-        <a:ext cx="6119640" cy="2699640"/>
+        <a:off x="7260120" y="7562880"/>
+        <a:ext cx="4319640" cy="2699640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2550,18 +3093,48 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>75</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>78120</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>128520</xdr:colOff>
-      <xdr:row>89</xdr:row>
-      <xdr:rowOff>32760</xdr:rowOff>
+      <xdr:row>64</xdr:row>
+      <xdr:rowOff>110880</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="3" name="Chart 4"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="14725800"/>
+        <a:ext cx="6119640" cy="2699640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>74</xdr:row>
+      <xdr:rowOff>78120</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>128520</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>110880</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 5"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -2570,7 +3143,7 @@
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2596,7 +3169,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 1"/>
+        <xdr:cNvPr id="5" name="Chart 1"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -2626,7 +3199,7 @@
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Chart 2"/>
+        <xdr:cNvPr id="6" name="Chart 2"/>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -2636,6 +3209,36 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>176040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>290880</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>187560</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Chart 3"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="12230280" y="571680"/>
+        <a:ext cx="3959640" cy="3059640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3179,6 +3782,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3343,49 +3947,98 @@
         <v>480</v>
       </c>
     </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J19" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="K19" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="L19" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J20" s="4" t="str">
+        <f aca="false">INDEX('Channel Composition'!$A$5:$A$7,MATCH(K20,'Channel Composition'!$B$5:$B$7,0))</f>
+        <v>Click and Collect</v>
+      </c>
+      <c r="K20" s="14" t="n">
+        <f aca="false">LARGE('Channel Composition'!$B$5:$B$7,1)</f>
+        <v>12557</v>
+      </c>
+      <c r="L20" s="15" t="n">
+        <f aca="false">K20/SUM('Channel Composition'!$B$5:$B$7)</f>
+        <v>0.354047424366312</v>
+      </c>
+    </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+      <c r="J21" s="4" t="str">
+        <f aca="false">INDEX('Channel Composition'!$A$5:$A$7,MATCH(K21,'Channel Composition'!$B$5:$B$7,0))</f>
+        <v>Delivery</v>
+      </c>
+      <c r="K21" s="14" t="n">
+        <f aca="false">LARGE('Channel Composition'!$B$5:$B$7,2)</f>
+        <v>11838</v>
+      </c>
+      <c r="L21" s="15" t="n">
+        <f aca="false">K21/SUM('Channel Composition'!$B$5:$B$7)</f>
+        <v>0.333775058505089</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>53</v>
+        <v>54</v>
+      </c>
+      <c r="J22" s="4" t="str">
+        <f aca="false">INDEX('Channel Composition'!$A$5:$A$7,MATCH(K22,'Channel Composition'!$B$5:$B$7,0))</f>
+        <v>In Store</v>
+      </c>
+      <c r="K22" s="14" t="n">
+        <f aca="false">LARGE('Channel Composition'!$B$5:$B$7,3)</f>
+        <v>11072</v>
+      </c>
+      <c r="L22" s="15" t="n">
+        <f aca="false">K22/SUM('Channel Composition'!$B$5:$B$7)</f>
+        <v>0.312177517128598</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="20" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -3394,50 +4047,70 @@
       <c r="F27" s="6"/>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J27" s="10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>51</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="J44" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="K44" s="22"/>
+      <c r="L44" s="22"/>
     </row>
     <row r="45" customFormat="false" ht="97.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B45" s="21" t="s">
-        <v>61</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="J45" s="22"/>
+      <c r="K45" s="22"/>
+      <c r="L45" s="22"/>
     </row>
     <row r="46" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="20" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B46" s="21" t="s">
-        <v>62</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="J46" s="22"/>
+      <c r="K46" s="22"/>
+      <c r="L46" s="22"/>
     </row>
     <row r="47" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="20" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B47" s="21" t="s">
-        <v>63</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="J47" s="22"/>
+      <c r="K47" s="22"/>
+      <c r="L47" s="22"/>
     </row>
     <row r="48" customFormat="false" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="20" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B48" s="21" t="s">
-        <v>64</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="J48" s="22"/>
+      <c r="K48" s="22"/>
+      <c r="L48" s="22"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B50" s="6"/>
       <c r="C50" s="6"/>
@@ -3448,63 +4121,64 @@
       <c r="H50" s="6"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="22" t="s">
-        <v>66</v>
+      <c r="A51" s="23" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="10" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A69" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="B69" s="23"/>
-      <c r="C69" s="23"/>
-      <c r="D69" s="23"/>
-      <c r="E69" s="23"/>
-      <c r="F69" s="23"/>
-      <c r="G69" s="23"/>
-      <c r="H69" s="23"/>
+      <c r="A69" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="22"/>
+      <c r="C69" s="22"/>
+      <c r="D69" s="22"/>
+      <c r="E69" s="22"/>
+      <c r="F69" s="22"/>
+      <c r="G69" s="22"/>
+      <c r="H69" s="22"/>
     </row>
     <row r="70" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="B70" s="23"/>
-      <c r="C70" s="23"/>
-      <c r="D70" s="23"/>
-      <c r="E70" s="23"/>
-      <c r="F70" s="23"/>
-      <c r="G70" s="23"/>
-      <c r="H70" s="23"/>
+      <c r="A70" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="22"/>
+      <c r="C70" s="22"/>
+      <c r="D70" s="22"/>
+      <c r="E70" s="22"/>
+      <c r="F70" s="22"/>
+      <c r="G70" s="22"/>
+      <c r="H70" s="22"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="10" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="23" t="s">
-        <v>71</v>
-      </c>
-      <c r="B73" s="23"/>
-      <c r="C73" s="23"/>
-      <c r="D73" s="23"/>
-      <c r="E73" s="23"/>
-      <c r="F73" s="23"/>
-      <c r="G73" s="23"/>
-      <c r="H73" s="23"/>
+      <c r="A73" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="B73" s="22"/>
+      <c r="C73" s="22"/>
+      <c r="D73" s="22"/>
+      <c r="E73" s="22"/>
+      <c r="F73" s="22"/>
+      <c r="G73" s="22"/>
+      <c r="H73" s="22"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="24" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
+    <mergeCell ref="J44:L48"/>
     <mergeCell ref="A69:H69"/>
     <mergeCell ref="A70:H70"/>
     <mergeCell ref="A73:H73"/>
@@ -3530,12 +4204,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Put student name and ID in their own rows on Start Here
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0122Czh11joCd8pnuPmWyXv4
</commit_message>
<xml_diff>
--- a/lab02/APIO114_Lab02_2713963.xlsx
+++ b/lab02/APIO114_Lab02_2713963.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="72">
   <si>
     <t xml:space="preserve">Lab 2 Chart Choice and Visual Design</t>
   </si>
@@ -31,7 +31,16 @@
     <t xml:space="preserve">APIO 114 Data Visualization | Semester 2027-01</t>
   </si>
   <si>
-    <t xml:space="preserve">Student: اروى حمدان الحربي  |  ID: 2713963</t>
+    <t xml:space="preserve">Student name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">اروى حمدان الحربي</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Student ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2713963</t>
   </si>
   <si>
     <t xml:space="preserve">Duration</t>
@@ -283,21 +292,14 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF222222"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -342,6 +344,13 @@
       <b val="true"/>
       <sz val="10"/>
       <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -402,15 +411,6 @@
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF17365D"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
         <color rgb="FFFFFFFF"/>
       </left>
@@ -428,7 +428,9 @@
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
-      <top/>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
@@ -437,9 +439,16 @@
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF17365D"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="FFD9D9D9"/>
       </bottom>
@@ -604,31 +613,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -692,11 +701,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -704,59 +713,59 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1062,11 +1071,11 @@
         </c:ser>
         <c:gapWidth val="55"/>
         <c:overlap val="0"/>
-        <c:axId val="40541759"/>
-        <c:axId val="46134616"/>
+        <c:axId val="56352799"/>
+        <c:axId val="89909192"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="40541759"/>
+        <c:axId val="56352799"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1099,7 +1108,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46134616"/>
+        <c:crossAx val="89909192"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1107,7 +1116,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="46134616"/>
+        <c:axId val="89909192"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1177,7 +1186,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40541759"/>
+        <c:crossAx val="56352799"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1385,11 +1394,11 @@
         </c:ser>
         <c:gapWidth val="55"/>
         <c:overlap val="0"/>
-        <c:axId val="19682116"/>
-        <c:axId val="80492597"/>
+        <c:axId val="18387022"/>
+        <c:axId val="12097278"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="19682116"/>
+        <c:axId val="18387022"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1422,7 +1431,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="80492597"/>
+        <c:crossAx val="12097278"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1430,7 +1439,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="80492597"/>
+        <c:axId val="12097278"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -1500,7 +1509,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19682116"/>
+        <c:crossAx val="18387022"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1931,11 +1940,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="50166213"/>
-        <c:axId val="70985252"/>
+        <c:axId val="67265759"/>
+        <c:axId val="60751017"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50166213"/>
+        <c:axId val="67265759"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1968,7 +1977,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="70985252"/>
+        <c:crossAx val="60751017"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1976,7 +1985,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="70985252"/>
+        <c:axId val="60751017"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="13000"/>
@@ -2021,7 +2030,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50166213"/>
+        <c:crossAx val="67265759"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2229,11 +2238,11 @@
         </c:ser>
         <c:gapWidth val="55"/>
         <c:overlap val="0"/>
-        <c:axId val="29310303"/>
-        <c:axId val="64952816"/>
+        <c:axId val="73928420"/>
+        <c:axId val="9868512"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="29310303"/>
+        <c:axId val="73928420"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2266,7 +2275,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64952816"/>
+        <c:crossAx val="9868512"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2274,7 +2283,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="64952816"/>
+        <c:axId val="9868512"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -2344,7 +2353,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29310303"/>
+        <c:crossAx val="73928420"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2756,61 +2765,71 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
+      <c r="B3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+    </row>
+    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>3</v>
+      <c r="A5" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>5</v>
+      <c r="A6" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>7</v>
+      <c r="A7" s="3" t="s">
+        <v>10</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>9</v>
+      <c r="A8" s="3" t="s">
+        <v>12</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>11</v>
+      <c r="A9" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -2821,14 +2840,14 @@
       <c r="H11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>16</v>
+      <c r="A12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2836,10 +2855,10 @@
         <v>1</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2847,10 +2866,10 @@
         <v>2</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2858,10 +2877,10 @@
         <v>3</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2869,10 +2888,10 @@
         <v>4</v>
       </c>
       <c r="B16" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="15" t="s">
         <v>21</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2880,10 +2899,10 @@
         <v>5</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -2930,7 +2949,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2938,35 +2957,35 @@
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="A5" s="3" t="s">
         <v>28</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B6" s="19" t="n">
         <v>6993.6</v>
@@ -2980,7 +2999,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B7" s="21" t="n">
         <v>6567</v>
@@ -2994,7 +3013,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B8" s="21" t="n">
         <v>11863.8</v>
@@ -3008,7 +3027,7 @@
     </row>
     <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B9" s="23" t="n">
         <v>10041.7</v>
@@ -3054,37 +3073,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>27</v>
+      <c r="A5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B6" s="19" t="n">
         <v>12556.6</v>
@@ -3095,7 +3114,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B7" s="21" t="n">
         <v>11837.7</v>
@@ -3106,7 +3125,7 @@
     </row>
     <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B8" s="23" t="n">
         <v>11071.8</v>
@@ -3151,7 +3170,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3169,7 +3188,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3186,29 +3205,29 @@
       <c r="N2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P4" s="25" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
@@ -3217,7 +3236,7 @@
       <c r="F5" s="26"/>
       <c r="G5" s="26"/>
       <c r="H5" s="26" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="I5" s="26"/>
       <c r="J5" s="26"/>
@@ -3225,11 +3244,11 @@
       <c r="L5" s="26"/>
       <c r="M5" s="26"/>
       <c r="N5" s="26"/>
-      <c r="P5" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q5" s="5" t="s">
-        <v>26</v>
+      <c r="P5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3359,14 +3378,14 @@
       <c r="L11" s="27"/>
       <c r="M11" s="27"/>
       <c r="N11" s="27"/>
-      <c r="P11" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q11" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="R11" s="5" t="s">
-        <v>44</v>
+      <c r="P11" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="R11" s="3" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3485,7 +3504,7 @@
       <c r="M16" s="27"/>
       <c r="N16" s="27"/>
       <c r="P16" s="28" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="Q16" s="29" t="n">
         <f aca="false">SUM('Channel Summary'!$B$6:$B$8)</f>
@@ -3508,7 +3527,7 @@
       <c r="M17" s="27"/>
       <c r="N17" s="27"/>
       <c r="P17" s="28" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="Q17" s="29" t="n">
         <f aca="false">SUM('Category Summary'!$B$6:$B$9)</f>
@@ -3531,7 +3550,7 @@
       <c r="M18" s="27"/>
       <c r="N18" s="27"/>
       <c r="P18" s="28" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="Q18" s="28" t="n">
         <f aca="false">SUM('Channel Summary'!$C$6:$C$8)</f>
@@ -3554,7 +3573,7 @@
       <c r="M19" s="27"/>
       <c r="N19" s="27"/>
       <c r="P19" s="28" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="Q19" s="28" t="n">
         <f aca="false">SUM('Category Summary'!$C$6:$C$9)</f>
@@ -3580,53 +3599,53 @@
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>50</v>
+      <c r="A23" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="139.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="31" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B24" s="32" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="33" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B25" s="34" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="33" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B26" s="34" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="84" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="35" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B27" s="36" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="37" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="H31" s="38" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="I31" s="38"/>
       <c r="J31" s="38"/>
@@ -3709,17 +3728,17 @@
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="37" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="39" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H50" s="40" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -3740,12 +3759,12 @@
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="41" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="38" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B68" s="38"/>
       <c r="C68" s="38"/>
@@ -3763,7 +3782,7 @@
     </row>
     <row r="69" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="38" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B69" s="38"/>
       <c r="C69" s="38"/>
@@ -3781,12 +3800,12 @@
     </row>
     <row r="71" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="41" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="38" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B72" s="38"/>
       <c r="C72" s="38"/>

</xml_diff>